<commit_message>
Add proposed 99-seat Sarawak demographic dataset
Same scrape applied to the SPR 2026 first-display proposal, which splits
the state's 887 polling districts into 1,141 across 99 DUN seats. The
82-seat workbook is regenerated from the shared builder so both files
carry identical structure and Read Me wording.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RvzGy6nkRN1PSRLyJ8WLZp
</commit_message>
<xml_diff>
--- a/data/sarawak-82-seats-demographics.xlsx
+++ b/data/sarawak-82-seats-demographics.xlsx
@@ -475,7 +475,7 @@
   <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -542,7 +542,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Sarawak — current 82 DUN seats / 31 Parlimen seats (state slug: 'sarawak', not the proposed redelineation 'sarawak-2026-p1')</t>
+          <t>Sarawak — current 82 DUN seats / 31 Parlimen seats (state slug: 'sarawak', the boundaries in force today)</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>The DUN/Parlimen sheets are aggregated in Python straight from the Polling Districts sheet's source rows (grouping by seat code and summing), not live Excel formulas — this sandbox's LibreOffice recalculation hung even on a single trivial formula, so live SUMIFS formulas could not be verified before shipping. The totals below are cross-checked against the state-wide totals during generation.</t>
+          <t>The DUN/Parlimen sheets are aggregated in Python straight from the Polling Districts sheet's source rows (grouping by seat code and summing), not live Excel formulas. Totals are cross-checked against the state-wide totals during generation.</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Roll-up to the 82 current state seats.</t>
+          <t>Roll-up to the 82 state seats.</t>
         </is>
       </c>
     </row>

</xml_diff>